<commit_message>
Added content to 03_DV_construction.qmd
</commit_message>
<xml_diff>
--- a/assets_output/03_DV_construction.xlsx
+++ b/assets_output/03_DV_construction.xlsx
@@ -1,38 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -40,18 +45,94 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -339,10 +420,233 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Table 3.1: Route outcomes after 3.08 years</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Route outcome</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Insecure outcome</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C3" t="n">
+        <v>38.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Returned to homelessness</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C4" t="n">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Independent accommodation</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>963</v>
+      </c>
+      <c r="C5" t="n">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Died</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>80</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Table 3.2: People with multiple returns during 7.5 yrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Multiple returns</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3460</v>
+      </c>
+      <c r="C10" t="n">
+        <v>92.09999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>295</v>
+      </c>
+      <c r="C11" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Table 3.3: People with a route in top 10% of route durations</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Had a longer-term route</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C15" t="n">
+        <v>86.59999999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="n">
+        <v>505</v>
+      </c>
+      <c r="C16" t="n">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Table 3.4: Returns within 2 years after moving to independent accommodation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Returned within 2y</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1022</v>
+      </c>
+      <c r="C20" t="n">
+        <v>97.7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>24</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added duration comparison to bivariate analysis (4)
</commit_message>
<xml_diff>
--- a/assets_output/03_DV_construction.xlsx
+++ b/assets_output/03_DV_construction.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="37">
   <si>
     <t>Table 3.1: Entry point into BAHSA services</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>Internal move: backwards</t>
+  </si>
+  <si>
+    <t>Insecure outcome (external)</t>
   </si>
 </sst>
 </file>
@@ -991,7 +994,7 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B57">
         <v>638</v>

</xml_diff>

<commit_message>
Updates to DVs and adding a DV as an IV.
</commit_message>
<xml_diff>
--- a/assets_output/03_DV_construction.xlsx
+++ b/assets_output/03_DV_construction.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
   <si>
     <t>Table 3.1: Entry point into BAHSA services</t>
   </si>
@@ -50,6 +50,54 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>Table 3.1.1: Entry point into BAHSA services (pathway and level)</t>
+  </si>
+  <si>
+    <t>pway_and_lvl</t>
+  </si>
+  <si>
+    <t>F L1</t>
+  </si>
+  <si>
+    <t>F L2</t>
+  </si>
+  <si>
+    <t>F L3</t>
+  </si>
+  <si>
+    <t>F L4</t>
+  </si>
+  <si>
+    <t>M L1</t>
+  </si>
+  <si>
+    <t>M L2</t>
+  </si>
+  <si>
+    <t>M L3</t>
+  </si>
+  <si>
+    <t>M L4</t>
+  </si>
+  <si>
+    <t>M/F L1</t>
+  </si>
+  <si>
+    <t>M/F L2</t>
+  </si>
+  <si>
+    <t>M/F L3</t>
+  </si>
+  <si>
+    <t>M/F L4</t>
+  </si>
+  <si>
+    <t>SU L1</t>
+  </si>
+  <si>
+    <t>SU L2</t>
   </si>
   <si>
     <t>Table 3.2: Route outcomes after 3.08 years</t>
@@ -482,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -615,10 +663,10 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>1148</v>
+        <v>255</v>
       </c>
       <c r="C13">
-        <v>34.4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -626,10 +674,10 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>1093</v>
+        <v>247</v>
       </c>
       <c r="C14">
-        <v>32.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -637,10 +685,10 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>1012</v>
+        <v>126</v>
       </c>
       <c r="C15">
-        <v>30.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -648,238 +696,272 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>80</v>
+        <v>221</v>
       </c>
       <c r="C16">
-        <v>2.4</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <v>3333</v>
+        <v>1308</v>
       </c>
       <c r="C17">
-        <v>100</v>
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18">
+        <v>78</v>
+      </c>
+      <c r="C18">
+        <v>1.5</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>18</v>
+      <c r="A19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19">
+        <v>50</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>2</v>
+        <v>21</v>
+      </c>
+      <c r="B20">
+        <v>520</v>
+      </c>
+      <c r="C20">
+        <v>10.3</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B21">
-        <v>1217</v>
+        <v>918</v>
       </c>
       <c r="C21">
-        <v>46.2</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B22">
-        <v>832</v>
+        <v>64</v>
       </c>
       <c r="C22">
-        <v>31.6</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B23">
-        <v>517</v>
+        <v>30</v>
       </c>
       <c r="C23">
-        <v>19.6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B24">
-        <v>66</v>
+        <v>176</v>
       </c>
       <c r="C24">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B25">
-        <v>2632</v>
+        <v>844</v>
       </c>
       <c r="C25">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>19</v>
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26">
+        <v>235</v>
+      </c>
+      <c r="C26">
+        <v>4.6</v>
       </c>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B28" s="1" t="s">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="B29">
-        <v>3460</v>
-      </c>
-      <c r="C29">
-        <v>92.09999999999999</v>
-      </c>
-    </row>
     <row r="30" spans="1:3">
-      <c r="A30" s="1" t="b">
-        <v>1</v>
+      <c r="A30" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="B30">
-        <v>295</v>
+        <v>1148</v>
       </c>
       <c r="C30">
-        <v>7.9</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="B31">
-        <v>3755</v>
+        <v>1093</v>
       </c>
       <c r="C31">
-        <v>100</v>
+        <v>32.8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>1012</v>
+      </c>
+      <c r="C32">
+        <v>30.4</v>
       </c>
     </row>
     <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>21</v>
+      <c r="A33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33">
+        <v>80</v>
+      </c>
+      <c r="C33">
+        <v>2.4</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="B35">
-        <v>3250</v>
-      </c>
-      <c r="C35">
-        <v>86.59999999999999</v>
+        <v>7</v>
+      </c>
+      <c r="B34">
+        <v>3333</v>
+      </c>
+      <c r="C34">
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:3">
-      <c r="A36" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B36">
-        <v>505</v>
-      </c>
-      <c r="C36">
-        <v>13.4</v>
+      <c r="A36" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37">
-        <v>3755</v>
-      </c>
-      <c r="C37">
-        <v>100</v>
+        <v>29</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38">
+        <v>1217</v>
+      </c>
+      <c r="C38">
+        <v>46.2</v>
       </c>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>23</v>
+      <c r="A39" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39">
+        <v>832</v>
+      </c>
+      <c r="C39">
+        <v>31.6</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>2</v>
+        <v>32</v>
+      </c>
+      <c r="B40">
+        <v>517</v>
+      </c>
+      <c r="C40">
+        <v>19.6</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B41">
-        <v>1022</v>
+        <v>66</v>
       </c>
       <c r="C41">
-        <v>97.7</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="B42">
-        <v>24</v>
+        <v>2632</v>
       </c>
       <c r="C42">
-        <v>2.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="1" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>1</v>
@@ -889,25 +971,25 @@
       </c>
     </row>
     <row r="46" spans="1:3">
-      <c r="A46" s="1" t="s">
-        <v>29</v>
+      <c r="A46" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="B46">
-        <v>762</v>
+        <v>3460</v>
       </c>
       <c r="C46">
-        <v>9</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="47" spans="1:3">
-      <c r="A47" s="1" t="s">
-        <v>30</v>
+      <c r="A47" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="B47">
-        <v>7708</v>
+        <v>295</v>
       </c>
       <c r="C47">
-        <v>91</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -915,7 +997,7 @@
         <v>7</v>
       </c>
       <c r="B48">
-        <v>8470</v>
+        <v>3755</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -923,12 +1005,12 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>1</v>
@@ -938,90 +1020,226 @@
       </c>
     </row>
     <row r="52" spans="1:3">
-      <c r="A52" s="1" t="s">
-        <v>33</v>
+      <c r="A52" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="B52">
-        <v>1562</v>
+        <v>3250</v>
       </c>
       <c r="C52">
-        <v>25.6</v>
+        <v>86.59999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:3">
-      <c r="A53" s="1" t="s">
-        <v>14</v>
+      <c r="A53" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="B53">
-        <v>1225</v>
+        <v>505</v>
       </c>
       <c r="C53">
-        <v>20.1</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="B54">
-        <v>1164</v>
+        <v>3755</v>
       </c>
       <c r="C54">
-        <v>19.1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B55">
-        <v>744</v>
-      </c>
-      <c r="C55">
-        <v>12.2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:3">
-      <c r="A56" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56">
-        <v>653</v>
-      </c>
-      <c r="C56">
-        <v>10.7</v>
+      <c r="A56" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B57">
-        <v>638</v>
-      </c>
-      <c r="C57">
-        <v>10.5</v>
+        <v>40</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="B58">
-        <v>117</v>
+        <v>1022</v>
       </c>
       <c r="C58">
-        <v>1.9</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59">
+        <v>24</v>
+      </c>
+      <c r="C59">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B63">
+        <v>762</v>
+      </c>
+      <c r="C63">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B64">
+        <v>7708</v>
+      </c>
+      <c r="C64">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B59">
+      <c r="B65">
+        <v>8470</v>
+      </c>
+      <c r="C65">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B69">
+        <v>1562</v>
+      </c>
+      <c r="C69">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B70">
+        <v>1225</v>
+      </c>
+      <c r="C70">
+        <v>20.1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B71">
+        <v>1164</v>
+      </c>
+      <c r="C71">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B72">
+        <v>744</v>
+      </c>
+      <c r="C72">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B73">
+        <v>653</v>
+      </c>
+      <c r="C73">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B74">
+        <v>638</v>
+      </c>
+      <c r="C74">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B75">
+        <v>117</v>
+      </c>
+      <c r="C75">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B76">
         <v>6103</v>
       </c>
-      <c r="C59">
+      <c r="C76">
         <v>100</v>
       </c>
     </row>

</xml_diff>